<commit_message>
feat: add calculate for incoming kanban stock order
</commit_message>
<xml_diff>
--- a/template_file/StockOutExportTemplate.xlsx
+++ b/template_file/StockOutExportTemplate.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\project-andum\Toho-Project\cmwi\backend\template_file\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38623CF7-5A0E-4664-B93E-CA88CC87699C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6CDE739-8E26-4BF9-AF48-35E3C52AF654}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="20370" yWindow="-4905" windowWidth="29040" windowHeight="15990" xr2:uid="{68B70A97-9B1A-4050-BAC0-10AB1B61C359}"/>
   </bookViews>
@@ -714,10 +714,10 @@
         <v>4</v>
       </c>
       <c r="E7" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="F7" s="7" t="s">
         <v>9</v>
-      </c>
-      <c r="F7" s="7" t="s">
-        <v>10</v>
       </c>
       <c r="G7" s="7" t="s">
         <v>5</v>

</xml_diff>

<commit_message>
refactor: change operator to requester in stock out export
</commit_message>
<xml_diff>
--- a/template_file/StockOutExportTemplate.xlsx
+++ b/template_file/StockOutExportTemplate.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\project-andum\Toho-Project\cmwi\backend\template_file\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\project-andum\cmwi\backend-cmw\template_file\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6CDE739-8E26-4BF9-AF48-35E3C52AF654}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBE1B372-CCB9-40C7-A4AA-E1A7C86F7DD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-4905" windowWidth="29040" windowHeight="15990" xr2:uid="{68B70A97-9B1A-4050-BAC0-10AB1B61C359}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{68B70A97-9B1A-4050-BAC0-10AB1B61C359}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,9 +39,6 @@
     <t>Code</t>
   </si>
   <si>
-    <t>Operator</t>
-  </si>
-  <si>
     <t>Quantity</t>
   </si>
   <si>
@@ -61,6 +58,9 @@
   </si>
   <si>
     <t>Stock Out</t>
+  </si>
+  <si>
+    <t>Requester</t>
   </si>
 </sst>
 </file>
@@ -629,7 +629,7 @@
   <sheetData>
     <row r="1" spans="1:14" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B1" s="11" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C1" s="11"/>
       <c r="D1" s="11"/>
@@ -666,7 +666,7 @@
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B4" s="12"/>
       <c r="C4" s="12"/>
@@ -684,7 +684,7 @@
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B5" s="13"/>
       <c r="C5" s="13"/>
@@ -711,19 +711,19 @@
         <v>3</v>
       </c>
       <c r="D7" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G7" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E7" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="F7" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="G7" s="7" t="s">
-        <v>5</v>
-      </c>
       <c r="H7" s="7" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I7" s="8"/>
     </row>

</xml_diff>